<commit_message>
UPDATE CODE AND EDIT SOME ISSUES
</commit_message>
<xml_diff>
--- a/VAS.xlsx
+++ b/VAS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Programing\-my projects-\chatTool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FC2BE5F-37F5-4247-B57A-A236483E8954}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{425C38EF-B166-4513-A2E8-28BD3F884D6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2550" yWindow="2550" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="174">
   <si>
     <t>Mobile Tracing</t>
   </si>
@@ -1892,6 +1892,27 @@
   </si>
   <si>
     <t>Description</t>
+  </si>
+  <si>
+    <t>CATIGORY</t>
+  </si>
+  <si>
+    <t>SERVICES</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> PORT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SIM&amp;LINE </t>
+  </si>
+  <si>
+    <t>Troubleshooting / INTERNET</t>
+  </si>
+  <si>
+    <t>Troubleshooting / SIM</t>
+  </si>
+  <si>
+    <t>Troubleshooting / Network</t>
   </si>
 </sst>
 </file>
@@ -2493,16 +2514,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="34.7109375" style="19" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="60.5703125" style="19" customWidth="1"/>
     <col min="3" max="3" width="46" style="19" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="9.140625" style="19"/>
+    <col min="4" max="4" width="17.140625" style="19" customWidth="1"/>
+    <col min="5" max="16384" width="9.140625" style="19"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:5">
       <c r="A1" s="20" t="s">
         <v>164</v>
       </c>
@@ -2512,8 +2534,11 @@
       <c r="C1" s="20" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="51">
+      <c r="D1" s="20" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="51">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -2524,10 +2549,13 @@
         <v>0</v>
       </c>
       <c r="D2" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="E2" s="18" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="63.75">
+    <row r="3" spans="1:5" ht="63.75">
       <c r="A3" s="18" t="s">
         <v>3</v>
       </c>
@@ -2538,10 +2566,13 @@
         <v>5</v>
       </c>
       <c r="D3" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="E3" s="18" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="51">
+    <row r="4" spans="1:5" ht="51">
       <c r="A4" s="18" t="s">
         <v>7</v>
       </c>
@@ -2552,10 +2583,13 @@
         <v>9</v>
       </c>
       <c r="D4" s="18" t="s">
+        <v>169</v>
+      </c>
+      <c r="E4" s="18" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="140.25">
+    <row r="5" spans="1:5" ht="140.25">
       <c r="A5" s="18" t="s">
         <v>11</v>
       </c>
@@ -2566,10 +2600,13 @@
         <v>13</v>
       </c>
       <c r="D5" s="18" t="s">
+        <v>169</v>
+      </c>
+      <c r="E5" s="18" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="140.25">
+    <row r="6" spans="1:5" ht="140.25">
       <c r="A6" s="18" t="s">
         <v>15</v>
       </c>
@@ -2580,10 +2617,13 @@
         <v>17</v>
       </c>
       <c r="D6" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="E6" s="18" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="382.5">
+    <row r="7" spans="1:5" ht="382.5">
       <c r="A7" s="18" t="s">
         <v>19</v>
       </c>
@@ -2594,10 +2634,13 @@
         <v>21</v>
       </c>
       <c r="D7" s="18" t="s">
+        <v>171</v>
+      </c>
+      <c r="E7" s="18" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="140.25">
+    <row r="8" spans="1:5" ht="140.25">
       <c r="A8" s="18"/>
       <c r="B8" s="2" t="s">
         <v>23</v>
@@ -2606,10 +2649,13 @@
         <v>24</v>
       </c>
       <c r="D8" s="18" t="s">
+        <v>171</v>
+      </c>
+      <c r="E8" s="18" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="255">
+    <row r="9" spans="1:5" ht="255">
       <c r="A9" s="18" t="s">
         <v>19</v>
       </c>
@@ -2620,10 +2666,13 @@
         <v>27</v>
       </c>
       <c r="D9" s="18" t="s">
+        <v>171</v>
+      </c>
+      <c r="E9" s="18" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="60">
+    <row r="10" spans="1:5" ht="60">
       <c r="A10" s="18" t="s">
         <v>29</v>
       </c>
@@ -2634,10 +2683,13 @@
         <v>31</v>
       </c>
       <c r="D10" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="E10" s="18" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="89.25">
+    <row r="11" spans="1:5" ht="89.25">
       <c r="A11" s="18" t="s">
         <v>29</v>
       </c>
@@ -2648,10 +2700,13 @@
         <v>34</v>
       </c>
       <c r="D11" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="E11" s="18" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="153">
+    <row r="12" spans="1:5" ht="153">
       <c r="A12" s="18" t="s">
         <v>36</v>
       </c>
@@ -2662,8 +2717,9 @@
         <v>38</v>
       </c>
       <c r="D12" s="18"/>
-    </row>
-    <row r="13" spans="1:4" ht="51">
+      <c r="E12" s="18"/>
+    </row>
+    <row r="13" spans="1:5" ht="51">
       <c r="A13" s="18" t="s">
         <v>39</v>
       </c>
@@ -2674,10 +2730,13 @@
         <v>41</v>
       </c>
       <c r="D13" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="E13" s="18" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="140.25">
+    <row r="14" spans="1:5" ht="140.25">
       <c r="A14" s="18" t="s">
         <v>43</v>
       </c>
@@ -2688,10 +2747,13 @@
         <v>45</v>
       </c>
       <c r="D14" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="E14" s="18" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="76.5">
+    <row r="15" spans="1:5" ht="76.5">
       <c r="A15" s="18" t="s">
         <v>47</v>
       </c>
@@ -2702,10 +2764,13 @@
         <v>49</v>
       </c>
       <c r="D15" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="E15" s="18" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="76.5">
+    <row r="16" spans="1:5" ht="76.5">
       <c r="A16" s="18" t="s">
         <v>51</v>
       </c>
@@ -2716,10 +2781,13 @@
         <v>53</v>
       </c>
       <c r="D16" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="E16" s="18" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="63.75">
+    <row r="17" spans="1:5" ht="63.75">
       <c r="A17" s="18" t="s">
         <v>55</v>
       </c>
@@ -2730,10 +2798,13 @@
         <v>57</v>
       </c>
       <c r="D17" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="E17" s="18" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="63.75">
+    <row r="18" spans="1:5" ht="63.75">
       <c r="A18" s="18" t="s">
         <v>59</v>
       </c>
@@ -2744,10 +2815,13 @@
         <v>61</v>
       </c>
       <c r="D18" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="E18" s="18" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="76.5">
+    <row r="19" spans="1:5" ht="76.5">
       <c r="A19" s="18" t="s">
         <v>63</v>
       </c>
@@ -2758,10 +2832,13 @@
         <v>65</v>
       </c>
       <c r="D19" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="E19" s="18" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="76.5">
+    <row r="20" spans="1:5" ht="76.5">
       <c r="A20" s="18" t="s">
         <v>67</v>
       </c>
@@ -2772,10 +2849,13 @@
         <v>69</v>
       </c>
       <c r="D20" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="E20" s="18" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="63.75">
+    <row r="21" spans="1:5" ht="63.75">
       <c r="A21" s="18" t="s">
         <v>71</v>
       </c>
@@ -2786,8 +2866,9 @@
         <v>73</v>
       </c>
       <c r="D21" s="18"/>
-    </row>
-    <row r="22" spans="1:4" ht="89.25">
+      <c r="E21" s="18"/>
+    </row>
+    <row r="22" spans="1:5" ht="89.25">
       <c r="A22" s="18" t="s">
         <v>74</v>
       </c>
@@ -2798,10 +2879,13 @@
         <v>76</v>
       </c>
       <c r="D22" s="18" t="s">
+        <v>172</v>
+      </c>
+      <c r="E22" s="18" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="76.5">
+    <row r="23" spans="1:5" ht="76.5">
       <c r="A23" s="1" t="s">
         <v>78</v>
       </c>
@@ -2812,10 +2896,13 @@
         <v>78</v>
       </c>
       <c r="D23" s="18" t="s">
+        <v>172</v>
+      </c>
+      <c r="E23" s="18" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="165.75">
+    <row r="24" spans="1:5" ht="165.75">
       <c r="A24" s="1" t="s">
         <v>81</v>
       </c>
@@ -2826,10 +2913,13 @@
         <v>81</v>
       </c>
       <c r="D24" s="18" t="s">
+        <v>172</v>
+      </c>
+      <c r="E24" s="18" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="63.75">
+    <row r="25" spans="1:5" ht="63.75">
       <c r="A25" s="1" t="s">
         <v>84</v>
       </c>
@@ -2840,10 +2930,13 @@
         <v>84</v>
       </c>
       <c r="D25" s="18" t="s">
+        <v>172</v>
+      </c>
+      <c r="E25" s="18" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="114.75">
+    <row r="26" spans="1:5" ht="114.75">
       <c r="A26" s="18" t="s">
         <v>87</v>
       </c>
@@ -2854,10 +2947,13 @@
         <v>89</v>
       </c>
       <c r="D26" s="18" t="s">
+        <v>172</v>
+      </c>
+      <c r="E26" s="18" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="51">
+    <row r="27" spans="1:5" ht="51">
       <c r="A27" s="18" t="s">
         <v>91</v>
       </c>
@@ -2867,11 +2963,14 @@
       <c r="C27" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D27" s="11" t="s">
+      <c r="D27" s="18" t="s">
+        <v>172</v>
+      </c>
+      <c r="E27" s="11" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="114.75">
+    <row r="28" spans="1:5" ht="114.75">
       <c r="A28" s="18" t="s">
         <v>94</v>
       </c>
@@ -2881,11 +2980,14 @@
       <c r="C28" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="D28" s="11" t="s">
+      <c r="D28" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="E28" s="11" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="63.75">
+    <row r="29" spans="1:5" ht="63.75">
       <c r="A29" s="18" t="s">
         <v>94</v>
       </c>
@@ -2895,11 +2997,14 @@
       <c r="C29" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="D29" s="11" t="s">
+      <c r="D29" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="E29" s="11" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="191.25">
+    <row r="30" spans="1:5" ht="191.25">
       <c r="A30" s="18" t="s">
         <v>101</v>
       </c>
@@ -2909,11 +3014,14 @@
       <c r="C30" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="D30" s="11" t="s">
+      <c r="D30" s="18" t="s">
+        <v>171</v>
+      </c>
+      <c r="E30" s="11" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="204">
+    <row r="31" spans="1:5" ht="204">
       <c r="A31" s="18" t="s">
         <v>105</v>
       </c>
@@ -2923,11 +3031,14 @@
       <c r="C31" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D31" s="11" t="s">
+      <c r="D31" s="18" t="s">
+        <v>171</v>
+      </c>
+      <c r="E31" s="11" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="255">
+    <row r="32" spans="1:5" ht="255">
       <c r="A32" s="18" t="s">
         <v>109</v>
       </c>
@@ -2937,11 +3048,14 @@
       <c r="C32" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="D32" s="11" t="s">
+      <c r="D32" s="18" t="s">
+        <v>171</v>
+      </c>
+      <c r="E32" s="11" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="51">
+    <row r="33" spans="1:5" ht="51">
       <c r="A33" s="8" t="s">
         <v>113</v>
       </c>
@@ -2951,9 +3065,12 @@
       <c r="C33" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="D33" s="18"/>
-    </row>
-    <row r="34" spans="1:4" ht="102">
+      <c r="D33" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="E33" s="18"/>
+    </row>
+    <row r="34" spans="1:5" ht="102">
       <c r="A34" s="8" t="s">
         <v>115</v>
       </c>
@@ -2963,9 +3080,12 @@
       <c r="C34" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="D34" s="18"/>
-    </row>
-    <row r="35" spans="1:4" ht="63.75">
+      <c r="D34" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="E34" s="18"/>
+    </row>
+    <row r="35" spans="1:5" ht="63.75">
       <c r="A35" s="8" t="s">
         <v>117</v>
       </c>
@@ -2975,9 +3095,12 @@
       <c r="C35" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="D35" s="18"/>
-    </row>
-    <row r="36" spans="1:4" ht="76.5">
+      <c r="D35" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="E35" s="18"/>
+    </row>
+    <row r="36" spans="1:5" ht="76.5">
       <c r="A36" s="13" t="s">
         <v>119</v>
       </c>
@@ -2988,10 +3111,13 @@
         <v>119</v>
       </c>
       <c r="D36" s="18" t="s">
+        <v>173</v>
+      </c>
+      <c r="E36" s="18" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="37" spans="1:4" ht="140.25">
+    <row r="37" spans="1:5" ht="140.25">
       <c r="A37" s="1" t="s">
         <v>122</v>
       </c>
@@ -3002,10 +3128,13 @@
         <v>122</v>
       </c>
       <c r="D37" s="18" t="s">
+        <v>173</v>
+      </c>
+      <c r="E37" s="18" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="38" spans="1:4" ht="178.5">
+    <row r="38" spans="1:5" ht="178.5">
       <c r="A38" s="18" t="s">
         <v>125</v>
       </c>
@@ -3016,8 +3145,9 @@
         <v>127</v>
       </c>
       <c r="D38" s="18"/>
-    </row>
-    <row r="39" spans="1:4" ht="153">
+      <c r="E38" s="18"/>
+    </row>
+    <row r="39" spans="1:5" ht="153">
       <c r="A39" s="1" t="s">
         <v>128</v>
       </c>
@@ -3027,11 +3157,14 @@
       <c r="C39" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="D39" s="11" t="s">
+      <c r="D39" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="E39" s="11" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="40" spans="1:4" ht="178.5">
+    <row r="40" spans="1:5" ht="178.5">
       <c r="A40" s="1" t="s">
         <v>131</v>
       </c>
@@ -3041,11 +3174,14 @@
       <c r="C40" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="D40" s="11" t="s">
+      <c r="D40" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="E40" s="11" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="41" spans="1:4" ht="191.25">
+    <row r="41" spans="1:5" ht="191.25">
       <c r="A41" s="1" t="s">
         <v>134</v>
       </c>
@@ -3055,11 +3191,14 @@
       <c r="C41" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="D41" s="11" t="s">
+      <c r="D41" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="E41" s="11" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="42" spans="1:4" ht="127.5">
+    <row r="42" spans="1:5" ht="127.5">
       <c r="A42" s="1" t="s">
         <v>137</v>
       </c>
@@ -3069,11 +3208,14 @@
       <c r="C42" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="D42" s="11" t="s">
+      <c r="D42" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="E42" s="11" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="43" spans="1:4" ht="63.75">
+    <row r="43" spans="1:5" ht="63.75">
       <c r="A43" s="6" t="s">
         <v>140</v>
       </c>
@@ -3084,8 +3226,9 @@
         <v>142</v>
       </c>
       <c r="D43" s="18"/>
-    </row>
-    <row r="44" spans="1:4" ht="77.25">
+      <c r="E43" s="18"/>
+    </row>
+    <row r="44" spans="1:5" ht="77.25">
       <c r="A44" s="1" t="s">
         <v>143</v>
       </c>
@@ -3096,8 +3239,9 @@
         <v>143</v>
       </c>
       <c r="D44" s="18"/>
-    </row>
-    <row r="45" spans="1:4" ht="114.75">
+      <c r="E44" s="18"/>
+    </row>
+    <row r="45" spans="1:5" ht="114.75">
       <c r="A45" s="18" t="s">
         <v>145</v>
       </c>
@@ -3107,11 +3251,14 @@
       <c r="C45" s="16" t="s">
         <v>147</v>
       </c>
-      <c r="D45" s="11" t="s">
+      <c r="D45" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="E45" s="11" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="46" spans="1:4" ht="76.5">
+    <row r="46" spans="1:5" ht="76.5">
       <c r="A46" s="8" t="s">
         <v>149</v>
       </c>
@@ -3121,11 +3268,14 @@
       <c r="C46" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="D46" s="11" t="s">
+      <c r="D46" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="E46" s="11" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="47" spans="1:4" ht="76.5">
+    <row r="47" spans="1:5" ht="76.5">
       <c r="A47" s="8" t="s">
         <v>152</v>
       </c>
@@ -3135,11 +3285,14 @@
       <c r="C47" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="D47" s="11" t="s">
+      <c r="D47" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="E47" s="11" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="48" spans="1:4" ht="76.5">
+    <row r="48" spans="1:5" ht="76.5">
       <c r="A48" s="8" t="s">
         <v>155</v>
       </c>
@@ -3149,11 +3302,14 @@
       <c r="C48" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="D48" s="11" t="s">
+      <c r="D48" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="E48" s="11" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="49" spans="1:4" ht="63.75">
+    <row r="49" spans="1:5" ht="63.75">
       <c r="A49" s="8" t="s">
         <v>158</v>
       </c>
@@ -3163,11 +3319,14 @@
       <c r="C49" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="D49" s="11" t="s">
+      <c r="D49" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="E49" s="11" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="50" spans="1:4" ht="45">
+    <row r="50" spans="1:5" ht="45">
       <c r="A50" s="8" t="s">
         <v>161</v>
       </c>
@@ -3177,7 +3336,10 @@
       <c r="C50" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="D50" s="11" t="s">
+      <c r="D50" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="E50" s="11" t="s">
         <v>163</v>
       </c>
     </row>

</xml_diff>